<commit_message>
update resource  mass maintenance
</commit_message>
<xml_diff>
--- a/data/Uploads/CustomerMaintenance.xlsx
+++ b/data/Uploads/CustomerMaintenance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Aishy QA\Robot Framework\Resona Spide\data\Uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9E7781-35D8-4ADE-8CFB-7C726DCEB654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDCDABF-CE84-43BA-979F-78DAF6F51C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3900" yWindow="2556" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>CIF No</t>
   </si>
@@ -75,23 +75,20 @@
     <t>Y</t>
   </si>
   <si>
-    <t>01602390-156</t>
-  </si>
-  <si>
-    <t>01693810-783</t>
-  </si>
-  <si>
-    <t>grenika@yahaa.com</t>
-  </si>
-  <si>
-    <t>jnebe@yahaa.com</t>
+    <t>01601150-156</t>
+  </si>
+  <si>
+    <t>01601150-157</t>
+  </si>
+  <si>
+    <t>hebas@yahaa.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,6 +107,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -583,7 +586,7 @@
         <v>17</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -788,6 +791,7 @@
       <c r="M19" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{C975109E-EB41-46E0-96EC-0429EBD03E0B}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{2BA3B85B-44A9-4EC7-9071-39247F2862DA}"/>

</xml_diff>